<commit_message>
feat: simplify Excel import template and fields by removing level, personal email, employee type, and status
</commit_message>
<xml_diff>
--- a/public/Humanius_Test_Personel_Listesi.xlsx
+++ b/public/Humanius_Test_Personel_Listesi.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,28 +413,19 @@
         <v>Departman</v>
       </c>
       <c r="E1" t="str">
-        <v>Pozisyon / Görev</v>
+        <v>Pozisyon</v>
       </c>
       <c r="F1" t="str">
-        <v>Kıdem Seviyesi</v>
+        <v>İşe Giriş Tarihi</v>
       </c>
       <c r="G1" t="str">
-        <v>İşe Giriş Tarihi</v>
+        <v>Kurumsal E-Posta</v>
       </c>
       <c r="H1" t="str">
-        <v>Kurumsal E-Posta</v>
+        <v>Telefon</v>
       </c>
       <c r="I1" t="str">
-        <v>Telefon</v>
-      </c>
-      <c r="J1" t="str">
         <v>Adres</v>
-      </c>
-      <c r="K1" t="str">
-        <v>İstihdam Türü</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Durum</v>
       </c>
     </row>
     <row r="2">
@@ -454,25 +445,16 @@
         <v>Kıdemli Frontend Geliştirici</v>
       </c>
       <c r="F2" t="str">
-        <v>Senior</v>
+        <v>2023-03-15</v>
       </c>
       <c r="G2" t="str">
-        <v>2023-03-15</v>
+        <v>kemal.kilic@humanius.net</v>
       </c>
       <c r="H2" t="str">
-        <v>kemal.kilic@humanius.net</v>
+        <v>05331112233</v>
       </c>
       <c r="I2" t="str">
-        <v>05331112233</v>
-      </c>
-      <c r="J2" t="str">
         <v>Kadıköy, İstanbul</v>
-      </c>
-      <c r="K2" t="str">
-        <v>normal</v>
-      </c>
-      <c r="L2" t="str">
-        <v>active</v>
       </c>
     </row>
     <row r="3">
@@ -492,25 +474,16 @@
         <v>İK ve Yetenek Uzmanı</v>
       </c>
       <c r="F3" t="str">
-        <v>Mid</v>
+        <v>2024-01-10</v>
       </c>
       <c r="G3" t="str">
-        <v>2024-01-10</v>
+        <v>selin.yilmaz@humanius.net</v>
       </c>
       <c r="H3" t="str">
-        <v>selin.yilmaz@humanius.net</v>
+        <v>05352223344</v>
       </c>
       <c r="I3" t="str">
-        <v>05352223344</v>
-      </c>
-      <c r="J3" t="str">
         <v>Beşiktaş, İstanbul</v>
-      </c>
-      <c r="K3" t="str">
-        <v>normal</v>
-      </c>
-      <c r="L3" t="str">
-        <v>active</v>
       </c>
     </row>
     <row r="4">
@@ -530,25 +503,16 @@
         <v>Kurumsal Satış Müdürü</v>
       </c>
       <c r="F4" t="str">
-        <v>Manager</v>
+        <v>2022-06-01</v>
       </c>
       <c r="G4" t="str">
-        <v>2022-06-01</v>
+        <v>burak.ozturk@humanius.net</v>
       </c>
       <c r="H4" t="str">
-        <v>burak.ozturk@humanius.net</v>
+        <v>05423334455</v>
       </c>
       <c r="I4" t="str">
-        <v>05423334455</v>
-      </c>
-      <c r="J4" t="str">
         <v>Çankaya, Ankara</v>
-      </c>
-      <c r="K4" t="str">
-        <v>normal</v>
-      </c>
-      <c r="L4" t="str">
-        <v>active</v>
       </c>
     </row>
     <row r="5">
@@ -568,30 +532,21 @@
         <v>Mali İşler Uzmanı</v>
       </c>
       <c r="F5" t="str">
-        <v>Senior</v>
+        <v>2021-11-20</v>
       </c>
       <c r="G5" t="str">
-        <v>2021-11-20</v>
+        <v>elif.cetin@humanius.net</v>
       </c>
       <c r="H5" t="str">
-        <v>elif.cetin@humanius.net</v>
+        <v>05554445566</v>
       </c>
       <c r="I5" t="str">
-        <v>05554445566</v>
-      </c>
-      <c r="J5" t="str">
         <v>Nilüfer, Bursa</v>
-      </c>
-      <c r="K5" t="str">
-        <v>normal</v>
-      </c>
-      <c r="L5" t="str">
-        <v>active</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>